<commit_message>
Add Russell Growth -> Value migration event study
- Members template now also builds a Russell 1000 Growth / Value workbook
- migration_universe.py finds stocks that leave RLG and land in RLV
  between snapshots and writes bbg/migration_events.csv
- bbg/build_migration_data_template.py turns those stocks plus sector
  benchmarks into a weekly BDH workbook
- migration_event_study.py measures return vs sector, EV/sales, forward
  P/E and implied vol from 52 weeks before to 52 weeks after, split by
  whether estimates were revised up or down beforehand

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018jgyEXzTPkofVxNMAUV9Bz
</commit_message>
<xml_diff>
--- a/bbg/bbg_index_members.xlsx
+++ b/bbg/bbg_index_members.xlsx
@@ -511,7 +511,7 @@
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Type Bloomberg index tickers and a peer group name in D11:E16 (yellow). Rows 11-14 are examples.</t>
+          <t>Type Bloomberg index tickers and a peer group name in D11:E16 (yellow). The filled rows are examples.</t>
         </is>
       </c>
     </row>
@@ -9479,7 +9479,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>Example indexes: S5HLTH = S&amp;P 500 Health Care, S5ENRS = Energy, S5INSU = Insurance, S5CONS = Consumer Staples. Confirm tickers on the index's DES page.</t>
+          <t>Example indexes: S5HLTH = S&amp;P 500 Health Care, S5ENRS = Energy, S5INSU = Insurance, S5CONS = Consumer Staples, RLG / RLV = Russell 1000 Growth / Value. Confirm tickers on the DES page.</t>
         </is>
       </c>
     </row>

</xml_diff>